<commit_message>
Auto-save blind test results via Streamlit
</commit_message>
<xml_diff>
--- a/盲測實驗結果.xlsx
+++ b/盲測實驗結果.xlsx
@@ -460,181 +460,181 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Salicylic Acid:當使用這個藥品，我該注意什麼?</t>
+          <t>Duratears:這藥可以幹嗎?</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1. 使用前請先告知醫師是否曾對水楊酸過敏或有肝臟、腎臟疾病、糖尿病、高血壓、消化性潰瘍等病史。2. 使用後若出現過敏現象如皮膚紅腫、發癢、呼吸困難等，請立即停藥並回診告知醫師。3. 若同時服用其他藥品，請告知醫師，以免發生藥物交互作用。4. 使用期間請避免日曬，外出時請做好防曬措施。5. 使用後若出現胃痛、噁心、嘔吐、下痢、食慾不振等症狀，請告知醫師。6. 使用後若出現皮膚脫皮、出血、感染等症狀，請立即停藥並回診告知醫師。</t>
+          <t>Duratears用於治療乾眼症。</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>若您有服用非類固醇抗發炎藥(NSAIDs)，請告知您的醫師，因為可能會增加副作用的機會。</t>
+          <t>Duratears用於治療乾眼症。</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>若您有任何過敏史、腎臟疾病、肝臟疾病、心臟病、高血壓、氣喘或其他呼吸問題、癲癇、糖尿病、消化性潰瘍、正在服用其他藥物、最近手術或傷口未愈者，請務必告知醫師您已知自己具有「葡萄糖耐受不佳」但尚未發展成為糖尿病的情況下，仍可使用此藥，但是需小心地監控您的血糖值果您已經知道您患有糖尿病，則須謹慎使用此藥品。</t>
+          <t>Duratears是一種治療乾眼症的藥物。它通過刺激淚腺分泌增加，從而改善眼睛乾澀不適的情況。此外，它還具有抗炎作用，可減輕眼部炎症。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nicotine: 我照顧的老人正在用這個藥有甚麼我要注意的嗎?</t>
+          <t>Fluticasone:使用這個藥品有可能會出現那些副作用?</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1. 請勿讓其他人使用您的藥品。2. 若您對尼古丁過敏或懷孕，請告知醫師。3. 若您正在服用下列藥品，請告知醫師：抗潰瘍劑、抗凝血劑、降血糖藥、制酸劑、避孕藥、抗癲癇藥、抗憂鬱劑、抗心律不整劑、β-阻斷劑、甲狀腺素、利尿劑、止痛劑、止咳劑、緩瀉劑、鈣離子阻斷劑。4. 若您有肝臟疾病、糖尿病、高血壓、心臟病、胃潰瘍、胃食道逆流、腎臟疾病、甲狀腺機能亢進、癲癇、青光眼、氣喘、肺氣腫、心律不整、中風、心肌梗塞、胸痛、心悸、頭痛、鼻炎、口腔潰瘍、腸阻塞、胃腸道出血、胃腸道穿孔、胰臟炎、肝炎、肝硬化、膽結石、腎功能低下、高血脂、高血鉀、高血鈉、低血鈣、高血壓、心衰竭、心肌纖維化、心肌缺血、心肌梗塞</t>
+          <t>頭痛. 咽喉炎. 鼻充血反跳現象. 鼻出血. 鼻腔感染(如: 鐵銹色鼻涕、嚴重鼻痛). 鼻腔刺激. 鼻腔潰瘍. 鼻腔過度生長. 鼻中隔穿孔. 鼻甲骨穿孔. 鼻中隔彎曲. 鼻甲骨萎縮. 鼻甲骨變窄.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>使用嗎啡長效膜衣錠時，應注意觀察是否產生藥物依賴性，特別是長期使用或高劑量使用時。對於老人，由於生理機能衰退，對藥物的反應可能會不同，因此使用時應小心，必要時應減量。</t>
+          <t>- 頭痛. 噁心. 鼻咽炎. 鼻充血反跳現象. 鼻出血. 鼻腔刺激. 鼻分泌物增加. 鼻腔念珠菌病(鵝口瘡).</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>如果您是幫助家人服藥，建議您留意家人的健康狀況，尤其是出現任何疑似「腎上腺功能不全」的非特定徵兆，如噁心、嘔吐、食欲下降、疲勞、昏厥、低血壓等，請儘快就醫，由醫師評估是否需要調整藥量或停止給藥。</t>
+          <t>頭痛、鼻炎、咽炎、咳嗽、喉嚨刺激、聲音嘶啞、口腔念珠菌感染(鵝口瘡)、耳鳴、心搏徐缓、低血糖、胰島素抗藥性、腹瀉、胃腸脹氣、消化不良、食慾減退、噁心、嘔吐、咽喉疼痛、顱内壓升高、眩暈、嗜睡、失眠、疲勞、發熱、背痛、肌肉痙攣、關節痛、肌膚紅疹、蕁麻疹、毛髮生長異位、男性乳房增大、女性陰道出血、月經週期改變、乳汁分泌、精子數目減少、白細胞減少、淋巴球減少、肝酶值上升、QT間期延長、房室結阻斷、無力、虛弱、呼吸困難、胸悶、支氣管收縮、哮喘惡化、急性呼吸道疾病、肺炎、肺栓塞、死亡。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Acetaminophen（Anti-phen）:我吃了 Anti-phen 退燒，但效果不好，可以自己增加劑量嗎？</t>
+          <t>Ibuprofen（Uprofen）:我頭痛想吃 Uprofen，但我本身有胃潰瘍病史，還能吃嗎？</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>不可以，請回診讓醫師評估。</t>
+          <t>如果您有嚴重肝腎疾病、腸胃道出血或對此藥過敏，請勿服用。若有下列情況，使用前請先告訴醫師：曾對此藥過敏、有氣喘、糖尿病、高血壓、心臟病、肝腎疾病、消化性潰瘍或正在服用其他藥物（特別是cyclosporin、dipyridamole、warfarin、methotrexate、lithium、ACE抑制劑、theophylline、probenecid、HIV藥物）果您有輕微的胃腸不適，可以和食物一起服用來降低胃腸方面的副作用。</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>不可以自行增加劑量，請回診告知醫師。</t>
+          <t>如果您有胃腸道疾病，如潰瘍或出血，請勿使用此藥。</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>不可以自行增減劑量，請回診告知醫師。</t>
+          <t>若您曾因胃腸道問題而停用 ibuprofen 或其他 NSAID，則不建議您再自行服藥。若有疑問，請詢問您的醫師或藥師。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Simethicone:如果忘記使用怎麼辦?</t>
+          <t>Sodium phosphate:使用這個藥品有可能會出現那些副作用?</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>想起時儘快服用，若已經接近下一次服藥時間，則跳過一次，依原來下一次的服藥時間服用即可，切勿一次服用兩倍劑量。</t>
+          <t>腹痛、腹脹、噁心、嘔吐、頭痛、暈眩、皮膚過敏。</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>想起時儘快服用，若已經接近下一次服藥時間，則跳過一次，依原來下一次的服用時間服用即可，切勿一次服用兩倍劑量。</t>
+          <t>腹痛、腹脹、噁心、嘔吐、頭痛、暈眩、虛弱、低血鈣、高血鉀、高血壓、低血壓、尿滯留、腸梗阻、腸穿孔、心律不整、心跳過速、呼吸困難、皮膚紅疹等。</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>想起時儘快服用，若已經接近下一次服藥時間，則跳過一次，依原來下一次的服用時間服用即可，切勿一次服用兩倍劑量。</t>
+          <t>腹瀉、噁心、嘔吐。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Urea: 這藥的作用機制是甚麼啊?我用起來皮膚很癢正常嗎?</t>
+          <t>Guaifenesin（Guaphen）:我痰很多，吃 Guaphen 後一直咳，是藥沒效嗎？</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>尿素軟膏用於治療濕疹、牛皮癬、燒傷、角化症等，其作用機制為促進表皮細胞之正常分化，並增加角質層水分含量而改善皮膚乾燥。使用後若出現皮膚癢感，可減少用量或間隔時間，若情況嚴重請告知醫師。</t>
+          <t>咳嗽是身體清除痰液的方式，服用本藥後可能會增加痰液排出，所以您會覺得一直在咳嗽，這不是藥物無效的現象。</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>尿素是一種軟化劑，可以增加頭皮的水分，使頭皮變得柔軟，從而幫助治療頭皮問題。當藥品中的尿素滲入頭皮時，它會降低頭皮表面的pH值，使頭皮變得更加柔軟，從而幫助治療頭皮問題。使用此藥後可能會出現輕微的皮膚刺激或搔癢感，但如果這種情況持續或加劇，請立即停藥並諮詢醫師。</t>
+          <t>咳嗽是身體清除痰液的方式之一，服用祛痰劑後，身體會增加排痰量，因此可能會更頻繁地咳嗽，這不是藥物無效的現象。</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>尿素軟膏具有角質溶解作用及保濕效果。當您擦上含有高濃度尿素成分之軟膏於患處時，由於其對表皮細胞具分解效應而使角質層變薄，因此可改善因角質增厚所引起的搔癢感；同時因為它能增加水分滯留能力，所以也能提高皮膚的含水量，從而達到治療目的。若您僅出現輕微的發癢現象，則屬於正常使用範圍內，但若您的情況持續惡化或是伴隨其它不適症状產生時，建議您儘速就診以獲得適當的指導。</t>
+          <t>不是。您服用了此藥後會有更多痰液產生，因此可能會更頻繁地咳嗽以清除痰液。這是一種正常反應，表示該藥對您的症狀有效果。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Nicotine:為什麼我要使用這個藥?</t>
+          <t>Simethicone:如果症狀完全好了，可以馬上停藥嗎？還是要把療程完成？</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -648,463 +648,460 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>尼古丁口錐可幫助戒除尼古丁成癮，減少抽菸次數或戒除抽菸。</t>
+          <t>如果症狀完全好了，建議繼續服藥一小時，再將劑量減半服用，之後再根據症狀改善情形調整治劑量或間隔時間，直到症狀完全消失。若症狀未完全消失，則需依照醫師指示服用至療程結束。</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>VEPESID用於治療某些類型的癌症，包括頑強性睪丸腫瘤、小細胞分化不良性肺癌、霍杰金氏症、非霍杰金氏惡性淋巴瘤、急性非淋巴細胞性白血病等。</t>
+          <t>如果您的消化不良症狀已經完全緩解，您可以考慮在當天結束時停止用藥。然而，如果您需要繼續按照醫生的指示完成整個療程，請遵照醫囑。</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>本藥品是一種輔助戒煙工具，可減輕您想抽菸時的不舒服感。它不會讓您恢復到正常吸菸狀態，但它會使您的身體感覺像是正在吸入一小撮煙霧一樣。這有助於緩解您想要重新開始抽菸的想法。</t>
+          <t>若您的症狀已經緩解，您可以考慮停止治療。然而，如果您希望確保所有症狀都已消退，最好按照醫師指示的整個療程進行治療。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Guaifenesin（Guaphen）:我痰很多，吃 Guaphen 後一直咳，是藥沒效嗎？</t>
+          <t>Benzydamine:當使用這個藥品，我該注意什麼?</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>咳嗽是身體清除痰液的方式，服用本藥後可能會增加痰液排出，所以您會覺得一直在咳嗽，這不是藥物無效的現象。</t>
+          <t>對此成份過敏者禁忌使用。本藥品不建議用於兒童及14歲以下青少年。本藥品僅適用於口腔局部治療，不可吞服或以吞服方式給藥。本藥品可能會使口腔黏膜變色，但不會影響其藥效。本藥品可能會使唾液變色，但不會影響其藥效。本藥品可能會使牙膏變色，但不會影響其藥效。本藥品可能會使假牙變色，若為白色假牙則會變色。</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>咳嗽是身體清除痰液的方式之一，服用祛痰劑後，可能會增加痰液的分泌，使痰液更容易排出，因此您可能會感覺到咳嗽的次數增加，這都是正常現象。但若您覺得咳嗽的症狀持續且嚴重，建議您回診與醫師討論。</t>
+          <t>對此成份過敏者禁忌使用。本藥不建議用於兒童及懷孕婦女。本藥可能會影響乳汁分泌，故哺乳婦女應避免使用。本藥可能會使唾液分泌減少，而增加口腔內細菌繁殖，因此建議飯後及睡前刷牙。</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>咳嗽症狀改善需要時間，建議持續服藥數天後再評估效果；若確實無任何療效，可向醫師諮詢其他可能的替代方案。</t>
+          <t>若您有下列情況，請告知您的醫師：曾對此藥過敏；同時服用其他藥物。您需要定期檢查血壓及心率。若出現以下嚴重不適之情形，應立即停藥並就診：呼吸困難、胸痛、發燒、喉嚨腫脹、皮膚疹等。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Simethicone:如果症狀完全好了，可以馬上停藥嗎？還是要把療程完成？</t>
+          <t>我口腔潰瘍發炎可以用什麼藥?</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>如果症狀完全好了，建議繼續服藥一小時，再將劑量減半服用，之後再根據症狀改善情形調整治劑量或間隔時間，直到症狀完全消失。若症狀未完全消失，則需依照醫師指示服用至療程結束。</t>
+          <t>可以使用含有類固醇的漱口水或口腔凝膠，如：Orabas 1000、Orabas 250、Orabas 500。</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>如果症狀完全好了，可以考慮停藥，但建議最好能完成整個療程，以確保療效。</t>
+          <t>口腔潰瘍發炎可以使用含有抗生素及類固醇的漱口水，如Orabas漱口水；或者使用局部性的消炎止痛劑，如潰可治軟膏。另外，維生素B群、C、Zinc等營養補充品也有助於潰瘍的癒合。</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>不可以立即停止服用，需按照醫師指示進行。</t>
+          <t>可以使用含有類固醇成分之漱口水或凝膠來消腫止痛；另外也可以局部外敷金霉素軟膏或紅汞(硫磺黴素)软膏来治療。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Diclofenac: 具體要儲存在多少度下?</t>
+          <t>Dextromethorphan:使用這個藥品有可能會出現那些副作用?</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>室溫儲存。</t>
+          <t>服用本藥時，若出現下列情況，請立即就醫：嚴重或持續的噁心、嘔吐、腹瀉、食慾不振、疲倦、虛弱、視覺模糊、頭痛、口乾、皮疹、昏睡、呼吸困難等。</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>請勿將Diclofenac儲存於超過30℃的環境。</t>
+          <t>服用此藥後可能會出現嗜睡、頭暈、口乾、噁心、嘔吐等現象，若情況嚴重或持續發生時請告知醫師。</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>對於不同形式的 Diclofenac，其儲存建議如下：
-- 凝膠：儲存溫度為 20°C 至 25°C （68°F 至 77°F），容許溫度波動範圍是 15°C 至 30°C （59°F 至 86°F）。請不要冷凍；避免受熱。
-- 解決液：儲存溫度上限為 25°C ，容許溫度波動範圍為15°C 到 30°C之間。
-- 紐扣式貼片：儲存溫度為 20°C 至 25°C （68°F 至 77°F），容許溫度波動範圍是 15°C 至 30°C （59°F 至 86°F）。不用時請保持封蓋緊閉。
-總結來說，大部分Diclafenac 的保存要求都是室溫即可，但為了確保品質，最好還是控制在較低溫度環境下存放。</t>
+          <t>服用此藥後可能會有嗜睡、頭暈等現象。若您發生過敏反應如搔癢、紅斑、呼吸困難；或是神經緊張、幻覺、噁心嘔吐、腹瀉、喉嚨痛、發燒、皮疹、虛弱無力、異常疲倦等症狀，應立即就醫。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Chlorhexidine:我該如何儲存這個藥品?</t>
+          <t>Acetaminophen:這個藥遇到哪些情況需要立刻停藥就醫？</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>室溫下緊密容器儲存。避免直接日照、熱、和溼氣。</t>
+          <t>對此成份過敏者。</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>請儲存於25℃以下。</t>
+          <t>對此藥過敏者，請立刻停藥，並告知醫師。出現皮膚疹、蕁麻疹、發癢、皮膚或眼睛變黃、關節腫痛、水腫、胸痛、呼吸短促、虛弱、手腳麻木、刺痛感等症狀，請立刻停藥，並告知醫師。</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>室溫保存(不超過30℃)，開封一個月即需丟棄不用。</t>
+          <t>如果您有肝臟疾病，應告知醫師。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Nicotine:當使用這個藥品，我該注意什麼?</t>
+          <t>Simethicone:如果忘記使用怎麼辦?</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1. 對尼古丁過敏者禁止使用。2. 使用本品前，若有下列事項請告知醫師：曾有藥物過敏、懷孕、哺乳、心臟血管疾病、腎臟疾病、肝臟疾病、消化性潰瘍、糖尿病、高血壓、甲狀腺機能亢進等病史或同時服用其他藥物（特別是cyclosporin、theophylline、diltiazem、disopyramide、verapamil） 3. 使用本品期間不可飲用含酒精性的飲料。4. 使用本品期間若出現下列異常情況時，應立即停藥並就醫：心律不整、心絞痛、心悸、胸痛、呼吸困難、噁心、嘔吐、皮膚紅疹、發癢、喉嚨痛、頭痛、暈眩、震顫、出汗、潮紅、顫抖、心神不定、焦慮、不安、情緒改變等。5. 使用本品期間不可進行吸煙戒斷治療。6. 使用本品期間不可進行吸煙戒斷治療。7. 使用本品期間不可進行吸煙戒斷治療。</t>
+          <t>想起時儘快服用，若已經接近下一次服藥時間，則跳過一次，依原來下一次的服藥時間服用即可，切勿一次服用兩倍劑量。</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>如果您正在使用尼古丁替代療法產品，請告知您的醫師。</t>
+          <t>想起時儘快服用，若已經接近下一次服藥時間，則跳過一次，依原來下一次的服藥時間服用即可，切勿一次服用兩倍劑量。</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>如果您正在吸煙，您應該盡快戒菸。這可能會使您的某些副作用更糟，並且可能會增加發生一些其他健康問題的可能性。請詢問醫師或其他醫療保健人員關於幫助您戒菸的選擇。</t>
+          <t>想起時儘快服用，若已經接近下一次服藥時間，則跳過一次，依原來下一次的服用時間服用即可，切勿一次服用兩倍劑量。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Choline Salicylate:使用這個藥品有可能會出現那些副作用?</t>
+          <t>Hydrocortisone:如果忘記使用怎麼辦?</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>過敏反應：皮膚紅腫、發癢、蕁麻疹、呼吸困難、喉嚨腫脹等。消化道：噁心、嘔吐、腹瀉、胃痛、食慾不振等。神經系統：頭痛、昏眩、嗜睡、失眠等。其他：發燒、皮疹、肝功能異常、血小板減少、血尿、皮膚黃疸等。</t>
+          <t>想起時儘快塗藥，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>過敏反應如皮疹、蕁麻疹、發癢、起泡或蕁麻疹；胸痛；呼吸短促；嘴唇、舌頭或喉嚨腫脹；臉部腫脹；嘴巴或喉嚨異常刺痛；聲音嘶啞；或呼吸困難。消化問題如腹瀉、嘔吐、胃痛或胃部不適。其他嚴重但罕見的副作用包括：肝臟問題（黃疸、尿色變深、胃痛、疲勞、噁心、嘔吐或食慾降低）。如果您出現任何黃疸或胃痛，請立即告知您的醫師。心律不整。若您感到心跳加速、心跳不規則、胸痛或呼吸短促，請立即致電您的醫師。體液滯留。若您感到頭暈、頭重腳輕、暈厥（失去知覺）、體重增加或呼吸困難，請立即致電您的醫師。</t>
+          <t>想起時儘快塗藥，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>過敏反應用藥品後感到搔癢、臉部或手部腫脹、嘴巴或喉嚨腫脹感或是呼吸困難等現象，請立即停藥並就醫果有以下情況，也請儘速告知醫生：皮膚疹、胃腸出血、耳鳴、眩暈、心跳加速或不規律、虛弱、意識不清、黃疸、嚴重嗜睡、視力改變、排尿困難等。</t>
+          <t>想起時儘快服用。但如果已接近下次給藥時間則跳過一次，依原來下一次的劑量給予即可。絕不可以一次给予兩倍劑量。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Simethicone:這個藥應該怎麼保存？開封後可以放多久？</t>
+          <t>Choline Salicylate:使用這個藥品有可能會出現那些副作用?</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>請存放於室溫下，避免陽光直射或潮濕環境，並置於兒童拿不到的地方。</t>
+          <t>過敏反應：皮膚紅腫、發癢、蕁麻疹、呼吸困難、喉嚨腫脹等。消化道：噁心、嘔吐、腹瀉、胃痛、食慾不振等。神經系統：頭痛、昏眩、嗜睡、失眠等。其他：發燒、皮疹、肝功能異常、血小板減少、血尿、皮膚黃疸等。</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>請置於兒童無法取得之處。儲存温度勿超過25°C若超過包裝所標示之有效期限，請勿再使用。使用完畢後，請妥善處理藥液匣。</t>
+          <t>過敏反應：皮膚紅腫、發癢、蕁麻疹、呼吸困難、喉嚨腫脹、嘴唇或舌頭腫脹等。消化系統：噁心、嘔吐、腹瀉、胃痛等。神經系統：頭痛、昏眩、嗜睡、焦慮等。其他：耳鳴、視力模糊、血尿、皮膚出血點、瘀青等。</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>室溫下避光存放；避免潮濕及陽光直曬。建議以原始容器包裝運送，可減少暴露於熱度和光照中。</t>
+          <t>過敏反應如皮疹、蕁麻疹、發癢、起紅腫。噁心、嘔吐、腹瀉等腸胃道症狀。頭痛、眩暈、耳鳴。肝功能異常。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Povidone Iodine: 孩子誤食了，會需要做什麼嗎?</t>
+          <t>Duratears:如果忘記使用怎麼辦?</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>若孩子誤食了，請立即就醫。</t>
+          <t>想起來時儘快使用。如果接近下次給藥時間則待下次給藥時間再使用，不需一次使用雙倍劑量。</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>誤食了Avelox，請立即就醫。</t>
+          <t>想起時儘快塗藥，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>如果孩子誤服了povidone碘，通常不需要特別處理，因為它是一種非毒性成分。但是，如果您有任何疑問或者孩子的狀況出現任何變化，如呼吸困難、嘔吐等症狀，請立即就醫。</t>
+          <t>想起時儘快塗藥，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Hydrocortisone:如果忘記使用怎麼辦?</t>
+          <t>Dextromethorphan（Medicon）:我最近感冒一直咳嗽，正在吃抗憂鬱藥，還能吃 Medicon 嗎？</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
         <v>1</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>想起時儘快塗藥，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。</t>
+          <t>若您有服用其他藥品，請事先告知醫師或藥師。若您有服用抗憂鬱藥，請先與醫師討論。</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>想起時儘快使用，若已經接近下一次服藥時間，則略過一次，依照原定時間用藥，不可一次使用雙倍劑量。</t>
+          <t>若您目前服用的抗憂鬱藥為三環類抗憂鬱藥，則不建議併用本品，以免增加心律不整之風險。但若您目前服用的抗憂鬱藥為SSRIs、SNRIs或其他非三環類抗憂鬱藥，則併用本品是安全的。</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>想起時儘快塗藥，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。若有任何疑問，請聯絡您的醫生尋求指示。</t>
+          <t>若您同時服用MAOI類抗憂鬱藥，則不建議併服此藥。若併服其他制酸劑(胃藥)，如含鋁之胃藥可能會降低本藥吸收量，故兩者應錯開至少二小時以上再服用。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Guaifenesin:用了多久還沒改善，就應該去看醫生？</t>
+          <t>Castor oil:為什麼我要使用這個藥?</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>若症狀持續超過7天，請諮詢醫師。</t>
+          <t>本藥可刺激腸道蠕動，用於緩解便秘或促進排便。</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>用藥後若症狀沒有改善，請於第7天後立即就醫。</t>
+          <t>Castor oil 通常用於緩解便秘。它通過刺激腸道運動來促進排便。</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>如果您的咳嗽持續了至少一個星期或者加重，您應該看醫生。如果您患有慢性阻塞性肺疾病(COPD)，哮喘或其他呼吸系統問題，請密切關注您的症状並定期看醫生。</t>
+          <t>本藥品是臨床常用於緩解偶發性便秘之症狀。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Castor oil:為什麼我要使用這個藥?</t>
+          <t>Povidone Iodine:忘記使用一次該怎麼辦？需要補用嗎？</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>本藥可刺激腸道蠕動，用於緩解便秘或促進排便。</t>
+          <t>想起時儘快塗藥，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Nexium屬於一種胃酸中和劑，可以減少胃酸分泌，適用於治療胃食道逆流疾病、十二指腸潰瘍等相關症狀。</t>
+          <t>想起時儘快塗藥，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Tolnaftate/ Methyl Salicylate/Pasca 是一種外用殺真菌劑，適用於治療各種形式的体癣、股癣和脚气。它通过抑制真菌细胞壁合成来发挥其杀菌作用。</t>
+          <t>若您錯過一劑，應儘快服用此藥。若您距離下一次預定服藥時間不到8小時，則跳過此次漏服劑量，在正常用藥時間繼續您的治療。切勿一次服用兩倍或額外劑量。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Acetaminophen:懷孕或哺乳期間可以使用這個藥嗎？</t>
+          <t>Choline Salicylate: 我突然牙齒來爆痛可以吃這個嗎?</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
         <v>2</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>可以使用，但請先諮詢醫師。</t>
+          <t>不可以，此藥主要是解熱鎮痛及抗發炎作用，並非治療牙齒疼痛。建議您儘快就醫，由牙醫師診治。</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>可以使用，但請先諮詢醫師或藥師。</t>
+          <t>牙齒疼痛可能由多種原因引起，包括蛀牙、牙髓炎、牙周病等。Choline Salicylate 主要用於退燒及止痛，並非專門治療牙齒疼痛的藥物。因此，如果您的牙齒突然出現爆痛，建議您儘快就診牙科醫生進行檢查，以確定疼痛的原因並接受適當的治療。
+同時，您可以使用含氟漱口水或冷熱開水漱口，以緩解牙齒疼痛。但請勿自行服用 Choline Salicylate 來治療牙齒疼痛，以免造成不必要的副作用或影響治療效果。</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>根據 Lexidrug 提供的信息，Povidone iodine 不適合用於懷孕或哺乳期間。對於此藥是否可以用於懷孕或哺乳，還需進一步確認其安全性。因此，在您懷孕或哺乳期間，最好避免自行使用此藥。</t>
+          <t>是的。您可以用此藥緩解牙痛，但最好還是去看牙医診治您的牙齒問題。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dextromethorphan:使用這個藥品有可能會出現那些副作用?</t>
+          <t>Magnesium Oxide: 小孩可以吃這個嗎?</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>服用本藥時，若出現下列情況，請立即就醫：嚴重或持續的噁心、嘔吐、腹瀉、食慾不振、疲倦、虛弱、視覺模糊、頭痛、口乾、皮疹、昏睡、呼吸困難等。</t>
+          <t>可以，但請先諮詢醫師或藥師。</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>頭痛、昏厥 (暈倒)、潮紅、低血壓、鼻道發炎 (鼻竇炎)、關節痛、心率不正常。</t>
+          <t>是的，小孩可以服用氧化鎂。氧化鎂是一種常見的通便劑，用於治療便秘或作為腸道準備手術前的清腸。但是，請遵照醫師指示使用，並確保兒童在成人監督下服用。</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>過敏反應用藥後感到疲倦想睡眩晕嘔吐噁心食慾減退</t>
+          <t>是的，小孩也可以食用此藥，但需依照醫師指示的劑量進行治療。</t>
         </is>
       </c>
     </row>
@@ -1118,13 +1115,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1133,328 +1130,330 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>請遵照醫師指示服用。</t>
+          <t>本藥為腸溶錠，通常一天服用兩次，飯後服用。請遵照醫師指示使用，一般建議每次服用1-2錠。</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>此藥通常由醫師指示使用，一般建議每日攝取約8克至10克，可搭配食物一起食用。但因您提供的信息主要關於Minoxidil，而 Magnesium Oxide 并未包含在此藥物列表中，所以無法確定是否需要配合此藥使用或是有特定的服藥方法。若您對此藥有任何疑問，請諮詢您的醫生。</t>
+          <t>請依照醫師指示服用。一般建議於飯後整粒吞服，勿咀嚼或咬碎膠囊。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Duratears:如果忘記使用怎麼辦?</t>
+          <t>Acetaminophen:懷孕或哺乳期間可以使用這個藥嗎？</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>想起來時儘快使用。如果接近下次給藥時間則待下次給藥時間再使用，不需一次使用雙倍劑量。</t>
+          <t>可以使用，但請先諮詢醫師。</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>想起時儘快服用，若已經接近下一次服藥時間，則跳過一次，依原來下一次的服用時間服用即可，切勿一次服用兩倍劑量。</t>
+          <t>可以使用，但請遵照醫師指示使用。</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>想起時盡快塗抹，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。</t>
+          <t>對於懷孕及哺乳女性，對乙酰氨基酚是一種較安全的選擇，但建議盡量減少用量並且不要超過必要的期限。另外，在研究中沒有明確顯示它會導致出生嬰兒發生先天異形或其他健康問題。因此，如果需要服用此類藥物，最好是在醫生指導下進行。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Choline Salicylate: 我突然牙齒來爆痛可以吃這個嗎?</t>
+          <t>Sodium phosphate／Disodium phosphate（Evac）:我已經好幾天沒排便了，可以一直用 Evac 幫助排便嗎？</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>不可以，此藥主要是解熱鎮痛及抗發炎作用，並非治療牙齒疼痛。建議您儘快就醫，由牙醫師診治。</t>
+          <t>不可以，超過三天未排便，請洽醫師。</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>牙齒疼痛可能由多種原因引起，包括蛀牙、牙髓炎、牙周病等。Moxifloxacin主要用於治療細菌感染，對於牙齒疼痛本身並無治療效果。因此，建議您儘快就診牙科醫生進行檢查，以確定牙齒疼痛的原因，並接受適當的治療。同時，如果您正在服用Moxifloxacin，請告知您的牙科醫生，以便她/他了解您的藥物使用情況。</t>
+          <t>不可以，使用時間請遵照醫師指示，一般建議使用一次即可。</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>不可以，您需要看牙科醫生診治您的疼痛原因。</t>
+          <t>不可以長期服用此類產品幫助排便，因為可能會造成腸道依賴性或其他副作用。如果您遇到排便困難的情況，建議您咨询醫生尋求適合您的治療方案。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Fluticasone:使用這個藥品有可能會出現那些副作用?</t>
+          <t>Hydrocortisone:我該如何使用這個藥?</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>頭痛. 咽喉炎. 鼻充血反跳現象. 鼻出血. 鼻腔感染(如: 鐵銹色鼻涕、嚴重鼻痛). 鼻腔刺激. 鼻腔潰瘍. 鼻腔過度生長. 鼻中隔穿孔.</t>
+          <t>遵照醫師指示使用。</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>頭痛、潮紅、低血壓、鼻竇炎、關節痛、心律不整等。</t>
+          <t>請遵照醫師指示使用。一般建議每日一次，皮膚外用。</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>- 頭痛- 心悸- 失眠- 口乾- 鼻咽炎- 上呼吸道感染- 鼻腔刺激- 鼻出血- 鼻息肉形成- 其他可能的副作用包括哮喘恶化、喉嚨痙攣、呼吸困難、胸悶、咳嗽及聲音嘶啞。如果您有上述任何情況，請立即就醫。</t>
+          <t>- 遵循醫師指示使用的頻率和方法。- 使用此藥之前，請務必洗手。- 將藥物塗抹於患處，避免擦掉。- 若您正在使用其他外用藥物，則需按照您的醫生指示的順序分別施用各藥物。- 在治療期間及停藥後的一段時間內，可能會出現反覆發癢的情況。若您感到任何不適，請告知您的醫生。</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Fluticasone（Flixonase）:鼻噴劑症狀改善後，還需要每天噴嗎？會不會有依賴性？</t>
+          <t>Dextromethorphan:我正在吃其他藥或保健食品，可以一起使用嗎？</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>即使症狀改善，仍需每天使用，以維持預防作用。並無成癮性。</t>
+          <t>若您正在服用其他藥品，請先告知醫師或藥師，以確保安全。</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>不需要每天噴，只有在症狀出現時才需要使用。且鼻噴劑不會產生依賴性。</t>
+          <t>若您正在服用其他藥品，請先告知醫師或藥師，以確保安全合併使用。</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>持續治療是為了預防反覆發作，而非僅止癥。因此即使症狀緩解了，也應該依照醫師指示繼續使用，不要自行停止。長期大量使用可能會產生依賴性，但短期使用則無須擔心。</t>
+          <t>若您現在服用任何藥物(包括非處方藥)，特別是抗抑郁劑、安眠藥等制吐劑、鎮靜劑及含有酒精成分之產品，請務必告知醫師。因為此類藥物可能會增加您對dextromethorphan 的敏感性而引發副作用；或者會降低dextromethorphan 在體內的濃度，影響治療效果。另外，若同時服用強效CYP2D6抑制劑者亦須小心。</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fluticasone: 肝功能有異常的兒童劑量藥多少?</t>
+          <t>Simethicone:這個藥應該怎麼保存？開封後可以放多久？</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26" t="n">
         <v>2</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1.5 mg/天</t>
+          <t>請存放於室溫下，避免陽光直射或潮濕環境，並置於兒童拿不到的地方。</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>請先諮詢醫師或藥師，以確保兒童使用安全。</t>
+          <t>請儲存在室溫下，避免潮濕或兒童可拿到的地方。</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>對於肝功能不全的小兒患者，建議調整劑量。具體劑量應由醫師根據病情評估後決定。</t>
+          <t>室溫下避光存放，保持乾燥，避免陽光直射。</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Betamethasone: 如果一直沒使用完，可以放多久還能用?</t>
+          <t>Ibuprofen:這藥是怎麼運作的</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>未開封前可存放於室溫下(30℃以下)，避免陽光直射。一旦打開包裝或放入冰箱，需在6週內使用完。</t>
+          <t>布洛芬是一種非類固醇抗發炎藥(NSAID)，具有解熱、止痛、抗發炎作用。</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>請勿使用超過標示之有效期限。</t>
+          <t>布洛芬是一種非類固醇抗發炎藥(NSAID)，它通過抑制體內發炎反應中的兩種酵素—環氧化酶-1(COX-1)和環氧化酶-2(COX-2)，來達到抗發炎、止痛及退燒的效果。</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>若超過標示之有效期限則不得使用；請存放於兒童接觸不到的地方。</t>
+          <t>本藥屬於非固醇抗發炎藥(NSAID)，它通過抑制身體產生發炎反應時所需要的兩種酵素(COX-1及COX-2)，而達到消炎止痛的效果。</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>8</v>
+        <v>58</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Diclofenac:我該如何使用這個藥?</t>
+          <t>Urea: 這藥的作用機制是甚麼啊?我用起來皮膚很癢正常嗎?</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
         <v>2</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>請遵照醫師指示及藥袋上之說明服用此藥藥期間請保留藥袋，以便即時獲取藥品資訊便症狀改善/病情穩定，仍應持續按照醫師指示服藥非醫師特別指示，此藥飯前或飯後服用皆可。</t>
+          <t>尿素軟膏用於治療濕疹、牛皮癬、燒傷、角化症等，其作用機制為促進表皮細胞之正常分化，並增加角質層水分含量而改善皮膚乾燥。使用後若出現皮膚癢感，可減少用量或間隔時間，若情況嚴重請告知醫師。</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>請遵照醫師指示使用。</t>
+          <t>尿素軟膏用於治療濕疹、牛皮癬、燒傷、角化症等，其作用機制主要是藉由提高角質層的含水量，使角質層柔軟化，並促進表皮細胞的正常更新。使用後可能會引起局部刺激或過敏反應，如皮膚發紅、乾燥、脫皮、刺痛或癢感等，這些症狀通常在短期內會消失。若症狀持續或加劇時，請告知醫師。</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>請依照醫師指示按時服用，一般是一天一次飯後服用。若您有任何疑問，請洽詢醫療人員。</t>
+          <t>尿素具有軟化角質層的效果，可以幫助去除表皮角質層的異常增生，因此對於某些皮膚疾病有療效。若您僅感到短期間的皮膚灼熱感或搔癢，則屬於正常現象，但若情況嚴重或持續時間較長，建議您回診讓醫師評估。</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Betamethasone:我該如何儲存這個藥品?</t>
+          <t>Crotamiton: 推薦我用這個藥的原因是甚麼?</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D29" t="n">
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>室溫下緊密容器儲存。避免直接日照、熱、和溼氣。</t>
+          <t>治療疥瘡、陰蝨感染。</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>請置於15~30℃，並置於孩童無法取得之處。</t>
+          <t>克他滿塗劑用於治療濕疹、皮膚炎、牛皮癬、燒傷、瘡口、皮膚潰瘍、皮膚感染、燒傷後疤痕、皮膚過敏、皮膚發癢症等。</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>室溫保存。請存放於兒童接觸不到的地方。</t>
+          <t>本藥品對於疥蟲具有良好的滅治效果，因此適用於治療疥瘡。此外，它也具備緩解搔癢的效果。</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Minoxidil:我該如何儲存這個藥品?</t>
+          <t>Diclofenac: 具體要儲存在多少度下?</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>室溫下儲存。</t>
+          <t>室溫儲存。</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>貯存於25°C以下。在儲存於8 °C以下時可能會發生沉澱。這種沉澱可在室溫下回溫時溶解。</t>
+          <t>室溫儲存。</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>室溫保存；避免陽光直射。</t>
+          <t>- 凝膠：儲存溫度為 20°C 至 25°C（68°F 至 77°F），允許溫度波動範圍為 15°C 至 30°C（59°F 至 86°F）。請勿冷凍；避免受熱。  
+- 結晶溶液：儲存在 25°C (77°F) 下；允許溫度在 15°C 至 30°C (59°F 至 86°F) 之間波動。  
+- 贏能軟膏：室溫保存即可。</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Hydrocortisone／Betamethasone:這個類固醇藥膏很有效，我可以一直擦到完全不癢嗎？</t>
+          <t>Duratears:我肝腎功能不好，可以使用嗎？</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1468,61 +1467,61 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>不可以，只可使用7天，超過7天可能有副作用發生。</t>
+          <t>若您有肝腎功能不全的情形，請告知您的醫師，由醫師評估是否適合使用。</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>不可以，因為皮膚對類固醇的耐受性有限，且長期使用會使皮膚變薄，增加感染風險，因此建議遵照醫師指示使用。</t>
+          <t>Duratears是一種人工淚液，用於乾眼症的治療。對於肝腎功能不佳的患者，一般來說是可接受的，但若有特殊劑型或用法需要考慮，請遵照醫師指示使用。</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>不可以。皮膚科醫師通常會指示您每天塗抹兩次，每次約半錢幣大小劑量，療程依病情而定，一般來說是7-14天。若您的症狀改善，仍應持續按照醫師指示使用的時間完成治療，以減少復發的機會。</t>
+          <t>Duratears 不建議對有嚴重肝臟疾病病史者及腎功能不全者使用。但對於一般情況下，若您的肝腎功能僅是輕微異常，則仍可正常使用；若您有任何疑問，請諮詢醫師意見。</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Minoxidil（Regaine）:擦 Regaine 後掉髮反而變多，是不是不適合我？</t>
+          <t>Povidone Iodine:這個藥要怎麼使用效果最好？一天要用幾次、用多久？</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>使用Regaine後，可能會有短暫的掉髮現象，通常在2-4週後會停止，此時再重新開始使用Regaine，效果會比未停用前更好。若掉髮現象持續超過4週，建議停用Regaine，待掉髮現象消失後再重新開始使用。</t>
+          <t>本藥品為外用消毒劑，通常建議每日使用2-3次，直到感染症狀消失。</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>使用Minoxidil後出現掉髮增多的情況，通常會在治療期間自然恢復。如果您對此有疑慮，建議您聯絡您的醫師進行討論。</t>
+          <t>本藥品通常用於外科手術前後、傷口清潔、皮膚消毒等。一般建議每日使用2-4次，每次使用量約10-20ml，將溶液浸泡雙手或傷口，至少浸泡1分鐘。</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>若您的頭髮在塗抹後數天至幾週內掉落，這可能是一種暫時性的現象，稱為「脫發期」，通常會持續約8-12周，在這個期間頭髮可能會比平常更多地掉落。然而，如果掉髮情況嚴重或持續時間超過預計，建議您停藥並諮詢醫師。</t>
+          <t>對於成人而言，povidone-碘可以用作口腔消毒劑。方法是每次漱口 10毫升，每日最多 4 次。另外，它也可以外用塗抹於患處，每日常規用量為 1至3次。</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Magnesium Oxide: 小孩可以吃這個嗎?</t>
+          <t>Povidone Iodine:這個藥有用吃的嗎?效果會不會比較好?</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1532,376 +1531,375 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>可以，但請先諮詢醫師或藥師。</t>
+          <t>Povidone Iodine並無口服劑型，僅有外用劑型。</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>可以，但請先諮詢醫師或藥師。</t>
+          <t>Povidone Iodine 通常不適用於口服，而是用於外用消毒。如果對碘過敏或有其他禁忌症時，請勿服用。</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>根據 Lexidrug 的數據，此藥不建議給予小於三個月大的嬰⼉。對於三個⽉以上的孩童，如果醫師認為其益處⾼過風險，則可以在醫師指導下服用。但通常情況下，除非有特殊需要，否則一般不會特別推薦给小孩服用。</t>
+          <t>不建議口服服用。僅可外用於皮膚或黏膜處。</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Benzydamine:當使用這個藥品，我該注意什麼?</t>
+          <t>Miconazole: 糖尿病患者有甚麼要注意的嗎?</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>對此成份過敏者禁忌使用。本藥品不建議用於兒童及14歲以下青少年。本藥品僅適用於口腔局部治療，不可吞服或以吞服方式給藥。本藥品可能會使口腔黏膜變色，但不會影響其藥效。本藥品可能會使唾液變色，但不會影響其藥效。本藥品可能會使牙膏變色，但不會影響其藥效。本藥品可能會使假牙變色，若為白色假牙則會變色。</t>
+          <t>使用本劑可能會引起低血糖，若同時服用降血糖藥物者，請告知醫師，以利評估您的治療方案。</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>使用此藥品時，請務必遵照醫師指示進行，並且要小心避免使用於眼睛四周、黏膜、濕疹或傷口等敏感部位。對於兒童使用，建議必須由保護者在監督下進行；而2歲以下的嬰兒則不建議自行使用，除非事先獲得醫師許可。此外，孕婦使用非類固醇抗發炎藥(NSAIDs)可能會對胎兒造成不良影響，因此孕婦不建議使用。</t>
+          <t>使用米康唑治療時，糖尿病患者應密切監測血糖水平，以避免可能的高血糖或低血糖問題。</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>- 使用此藥品之前，如果您患有胃潰瘍或其他消化道疾病、肝病、腎病、糖尿病、高血壓、甲狀腺機能亢進、青光眼、氣喘、前列腺肥大、心律失調、精神障礙、免疫系統問題或正在接受放療/化疗，請務必告知醫生。- 若您正服用下列藥品，也請告訴您的醫生：阿斯匹靈、布洛芬、消炎痛、強力霉素、磺胺劑、HIV/AIDS藥物、利多卡因凝膠、碘酒、鈉氯化物注射液、苯妥英錠、地西泮片、普魯卡因胺錠、奎尼丁錠、三環抗 depressant、cyclosporin、dexamethasone、fluconazole、itraconoz
-- 在使用此藥品期間以及停藥後的一周內，請做好防晒措施以防止發生光敏感現象。- 如果您是懷孕或計畫懷孕，請讓醫生知道。- 喂食嬰幼兒的母親若想使用此藥品，則需事先諮詢醫生。</t>
+          <t>提醒糖尿病患者需定期監測血糖值，以確保安全。</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Acetaminophen:這個藥遇到哪些情況需要立刻停藥就醫？</t>
+          <t>Ibuprofen: 可以和Diclofenac同時使用嗎?</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
         <v>1</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>對此成份過敏者。</t>
+          <t>不可以，兩種藥物都屬於非類固醇抗發炎藥(NSAID)，不建議同時服用。</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>對此成份過敏者，請立刻停藥就醫。</t>
+          <t>不可以，兩種藥物都屬於非類固醇抗發炎藥(NSAID)，不建議同時服用，以免造成肝臟損害。</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>對此成份過敏者，請告知醫師。</t>
+          <t>不可以。建議您只選擇其中一種非類固醇抗發炎藥服用即可。若您有其他疾病需要併服其他的非類固醇抗發炎藥也請告訴您的醫師。</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Amorolfine:我該如何使用這個藥?</t>
+          <t>Cough Mixture 2:咳嗽糖漿喝了很想睡，白天還能繼續喝嗎？</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>遵照醫師指示使用。</t>
+          <t>可以，但請注意白天服用此藥後若感到嗜睡，請勿從事容易引起傷害的危險活動，如開車、操作機械等。</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>請遵照醫師指示使用。</t>
+          <t>可以，但請注意不要開車或操作危險機械等需要精神集中的工作或活動。</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>塗抹患部皮膚上，待其乾燥即可。</t>
+          <t>若您服用了大量的本藥品，可能會出現嗜睡現象，但通常不會影響您白天的工作或生活。若您的症狀持續數日無法緩解，則需回診讓醫師評估您的情況。</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Ibuprofen（Uprofen）:我頭痛想吃 Uprofen，但我本身有胃潰瘍病史，還能吃嗎？</t>
+          <t>Hydrocortisone／Betamethasone:這個類固醇藥膏很有效，我可以一直擦到完全不癢嗎？</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" t="n">
         <v>2</v>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>如果您有嚴重肝腎疾病、腸胃道出血或對此藥過敏，請勿服用。若有下列情況，使用前請先告訴醫師：曾對此藥過敏、有氣喘、糖尿病、高血壓、心臟病、肝腎疾病、消化性潰瘍或正在服用其他藥物（特別是cyclosporin、dipyridamole、warfarin、methotrexate、lithium、ACE抑制劑、theophylline、probenecid、HIV藥物）果您有輕微的胃腸不適，可以和食物一起服用來降低胃腸方面的副作用。</t>
+          <t>不可以，只可使用7天，超過7天可能有副作用發生。</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>如果您有胃腸道疾病，建議您在使用非類固醇抗發炎藥前，先告知醫師，以利醫師為您選擇適合的藥品。</t>
+          <t>不可以，因為皮膚對此類藥物會產生抗性，所以不可長期使用。</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>若您曾因服用非類固醇抗發炎藥出現消化性潰瘍或腸道出血的情形，則不建議您再服用了。另外如果您同時患有肝臟疾病、腎臟疾病或有該病史、支气管哮喘、高血壓，也應告知醫師以利評估是否適合給藥。</t>
+          <t>不可以哦！雖然這種藥膏對濕疹、牛皮廬、燒傷、割傷、搔抓過敏及接觸性皮膚炎都有很好的緩解效果，但您僅需按照醫師指示使用的次數即可，通常是一天兩次，而且一定要持續觀察您的病情，當症狀改善時就要停止使用，否則可能會造成副作用發生。另外，也不建議自行增減用量或是停藥，最好能回診讓醫師評估喔！</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Miconazole:使用這個藥品有可能會出現那些副作用?</t>
+          <t>Nicotine（Nicorette／Smokfree）:我抽菸的同時使用戒菸口香糖，這樣會不會有問題？</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" t="n">
         <v>2</v>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>皮膚刺激、搔癢、紅斑、發疹、頭痛、噁心、嘔吐、腹瀉、胃部不適等。</t>
+          <t>不建議在抽菸時使用戒菸口香糖，因為這兩種產品都是為了緩解戒斷症狀而設計的，如果同時使用可能會造成過度刺激。</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>頭痛、潮紅、低血壓、鼻竇炎、關節痛、心率不正常等。</t>
+          <t>同時使用尼古丁口香糖和尼古丁吸入劑可能會增加尼古丁的吸收，因此不建議同時使用兩種尼古丁替代療法。如果您已經開始使用一種尼古丁替代療法，請先告知您的醫師，以評估是否適合開始使用另一種尼古丁替代療法。</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>皮膚刺激、搔癢、皮疹、黏膜灼熱感、呼吸困難、喉嚨緊繃、咳嗽、聲音嘶啞、吞嚥困難、舌頭變色等。</t>
+          <t>不可以同時抽菸以及使用尼古丁口香糖，因為這兩種方式都會讓您得到相同的刺激感，而無法達到戒除菸癮的目的。所以當您想要使用尼古丁口香糖的時候，就要把手中的菸丟掉，並且盡快地含住口香糖，直到感覺到口中有一股苦味，此時就代表口香糖已經釋放出尼古丁了，接著再咀嚼口香糖，一直到苦味消失即可，之後每隔一小時換新的口香糖，如此持續至醫生指示之時間止。</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Povidone Iodine:優碘是不是擦越多越好？傷口每天都要消毒嗎？</t>
+          <t>Guaifenesin:哪些症狀代表可能不是小問題，而是需要盡快就醫？</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D39" t="n">
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>擦太多會使皮膚過於乾燥，且對皮膚有刺激性。傷口每天不需要消毒，但若有分泌物或感染時則需適當清潔。</t>
+          <t>若出現下列情況時，請立即就醫：1. 持續的咳嗽或呼吸困難。2. 頭痛、暈眩或意識混亂。3. 胸痛或胸悶。4. 心跳加速或不規則。5. 皮膚或眼睛發黃（黃疸）。6. 皮膚疹或其他過敏反應。7. 出血或瘀傷。8. 離奇的虛弱或疲倦。</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>使用優碘時，建議遵照醫師指示進行消毒，通常建議每日一次，塗抹於患部表面，以達到清潔的效果。但也不需要過量使用，因為過多的碘可能對皮膚造成刺激。</t>
+          <t>咳嗽持續不緩解或加重，伴隨呼吸困難、胸痛、發燒等症狀，應儘速就醫。</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>不是的，您只需依照醫師指示進行清潔即可。</t>
+          <t>若出現過敏反應如發燒、喉嚨痛、臉部或手部腫脹、嘴巴或舌頭起泡、呼吸困難等症狀，應立即停藥並尋求醫師幫助。</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Dextromethorphan（Medicon）:我最近感冒一直咳嗽，正在吃抗憂鬱藥，還能吃 Medicon 嗎？</t>
+          <t>Salicylic Acid:當使用這個藥品，我該注意什麼?</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
         <v>2</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>若您有服用其他藥品，請事先告知醫師或藥師。若您有服用抗憂鬱藥，請先與醫師討論。</t>
+          <t>1. 使用前請先告知醫師是否曾對水楊酸過敏或有肝臟、腎臟疾病、糖尿病、高血壓、消化性潰瘍等病史。2. 使用後若出現過敏現象如皮膚紅腫、發癢、呼吸困難等，請立即停藥並回診告知醫師。3. 若同時服用其他藥品，請告知醫師，以免發生藥物交互作用。4. 使用期間請避免日曬，外出時請做好防曬措施。5. 使用後若出現胃痛、噁心、嘔吐、下痢、食慾不振等症狀，請告知醫師。6. 使用後若出現皮膚脫皮、出血、感染等症狀，請立即停藥並回診告知醫師。</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>若您目前正服用抗憂鬱藥，請先告知您的醫師，由醫師評估是否適合併用。</t>
+          <t>對水楊酸過敏者禁止使用；患有肝、腎、腸胃障礙及支氣管氣喘者，應謹慎使用。避免同時服用阿斯匹靈及其他含水楊酸之藥品及酒精性飲料。此藥會使皮膚對日光敏感，應避免陽光直接照射。此藥可能會影響某些化驗結果，如尿液中的葡萄糖含量。</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>若您有下列情況，請勿服用此藥：曾因服用MAOIs(三環抗忧鬱劑)而發生過嚴重的高血壓反應；懷孕或哺乳期女性；癲癇病史患者；青光眼患者；排尿困難; 避免飲酒, 若服用了含有酒精成分之製劑如止咳糖漿等也需避免。</t>
+          <t>若您對水楊酸過敏或者您正在服用其他含有水楊酸成分的非處方止痛消炎劑(如阿斯匹靈)，請告知醫師。若您的肝臟或腎臟功能不佳，也應告訴醫師。另外如果有胃潰瘍病史或是消化道容易出血者，也不適合使用此藥。</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Amorolfine（Loceryl Nail Lacquer）:灰指甲擦了兩個月都沒好，是不是沒效？還要擦多久？</t>
+          <t>Minoxidil（Regaine）:擦 Regaine 後掉髮反而變多，是不是不適合我？</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41" t="n">
         <v>3</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>治療灰指甲通常需要較長時間，一般建議治療至少6個月以上。因此，您目前使用兩個月並未見療效，這可能是正常情況。請繼續按照醫師指示進行治療，不要自行停藥或更改劑量。</t>
+          <t>使用Regaine後，可能會有短暫的掉髮現象，通常在2-4週後會停止，此時再重新開始使用Regaine，效果會比未停用前更好。若掉髮現象持續超過4週，建議停用Regaine，待掉髮現象消失後再重新開始使用。</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>治療灰指甲通常需要較長時間的治療，一般建議至少6個月以上。若您已經使用兩個月仍未見改善，建議您回診與醫師討論，以評估是否需要調整治療方案。</t>
+          <t>使用Regaine後，可能會有一段時間頭髮會變得比較稀疏，這是一種暫時性的現象，之後頭髮會逐漸恢復正常。但如果使用後頭髮變得更多，這可能表示您對這種藥物不適合，建議停用並詢問醫師。</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>治療時間因人而異，通常需要數週至數個月。若您的病情未改善，建議諮詢醫師。</t>
+          <t>有可能是您對此成分過敏或是不适合使用該藥物，建議停藥並回診告知醫師。</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Urea:為什麼我要使用這個藥?</t>
+          <t>Cough Mixture:為什麼我要使用這個藥?</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>此藥用於治療高血漿尿素氮症，通常發生於腎臟病患者。</t>
+          <t>本藥品是化痰劑，可以幫助排痰。</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Aromasin用於具有雌激素受體陽性之停經婦女，使用Tamoxifen至少兩年之早期侵犯性乳癌的輔助治療。Aromasin用於已接受抗雌激素而無效之停經婦女晚期乳癌。</t>
+          <t>止咳糖漿用於緩解咳嗽症状。</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>此藥用於控制嚴重嘔吐及噁心。</t>
+          <t>本藥品是針對咳嗽以及上呼吸道過敏所引起之相關症狀(如：流鼻水、打噴涕等)，具有暫時緩解的作用。</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Povidone Iodine:忘記使用一次該怎麼辦？需要補用嗎？</t>
+          <t>Guaifenesin:用了多久還沒改善，就應該去看醫生？</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>想起時儘快塗藥，若已接近下一次用藥時間則略過一次，依照原定時間用藥，絕不可一次使用兩倍劑量。</t>
+          <t>若症狀持續超過7天，請諮詢醫師。</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>當想起時趕快服藥，若想起時已接近下次服用時間，則不須服藥，等到下次該吃藥時再服藥即可，但千萬不可一次服用兩倍的劑量。</t>
+          <t>如果您的咳嗽持續超過7天，或者您的症狀沒有改善，請儘快就醫。</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>想起時儘快塗擦，如果接近下次給藥時間則待下次給藥時間再使用，不需一次使用雙倍劑量。</t>
+          <t>如果症狀持續超過7天未見緩解，或者出現呼吸困難、胸痛等情況，請儘速就診。</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Guaifenesin:哪些症狀代表可能不是小問題，而是需要盡快就醫？</t>
+          <t>Miconazole:使用這個藥品有可能會出現那些副作用?</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
         <v>1</v>
@@ -1911,173 +1909,173 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>若出現下列情況時，請立即就醫：1. 持續的咳嗽或呼吸困難。2. 頭痛、暈眩或意識混亂。3. 胸痛或胸悶。4. 心跳加速或不規則。5. 皮膚或眼睛發黃（黃疸）。6. 皮膚疹或其他過敏反應。7. 出血或瘀傷。8. 離奇的虛弱或疲倦。</t>
+          <t>皮膚刺激、搔癢、紅斑、發疹、頭痛、噁心、嘔吐、腹瀉、胃部不適等。</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>若出現呼吸急促、呼吸困難、發燒、喉嚨痛、耳朵痛、頭痛、皮膚疹、皮膚或眼睛變黃、血尿、關節痛、虛弱、疲倦、異常出血、瘀青、皮膚或眼睛顏色改變、視力改變、耳鳴、心跳過快或心跳異常、手腳麻木或刺痛、口乾、肌肉疼痛、發抖、無法站立或行走、異常的感覺或行為、憂鬱、意識惑亂、吞嚥困難、皮膚過敏反應等症狀時，請立即就醫。</t>
+          <t>皮膚刺激、搔癢、紅斑、發疹、頭痛、噁心、嘔吐、腹瀉、胃腸不適。</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>若出現以下情況，請立即停藥並尋求醫師幫助：嚴重嗜睡、頭昏眼花、幻覺、運動困難等。</t>
+          <t>皮膚刺激感。</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Sodium phosphate／Disodium phosphate（Evac）:我已經好幾天沒排便了，可以一直用 Evac 幫助排便嗎？</t>
+          <t>Nicotine:當使用這個藥品，我該注意什麼?</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>不可以，超過三天未排便，請洽醫師。</t>
+          <t>1. 對尼古丁過敏者禁止使用。2. 使用本品前，若有下列事項請告知醫師：曾有藥物過敏、懷孕、哺乳、心臟血管疾病、腎臟疾病、肝臟疾病、消化性潰瘍、糖尿病、高血壓、甲狀腺機能亢進等病史或同時服用其他藥物（特別是cyclosporin、theophylline、diltiazem、disopyramide、verapamil） 3. 使用本品期間不可飲用含酒精性的飲料。4. 使用本品期間若出現下列異常情況時，應立即停藥並就醫：心律不整、心絞痛、心悸、胸痛、呼吸困難、噁心、嘔吐、皮膚紅疹、發癢、喉嚨痛、頭痛、暈眩、震顫、出汗、潮紅、顫抖、心神不定、焦慮、不安、情緒改變等。5. 使用本品期間不可進行吸煙戒斷治療。6. 使用本品期間不可進行吸煙戒斷治療。7. 使用本品期間不可進行吸煙戒斷治療。</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>不可以，超過建議使用天數可能會造成腸道功能障礙，導致長期便秘。</t>
+          <t>戒菸過程中可能會出現一些不適感，如焦慮、失眠、頭痛、噁心、腹瀉、口乾、流汗、咳嗽、喉嚨痛、鼻塞、打噴嚏、味覺改變、異常口渴、異常食慾等，通常在服藥一段時間後會改善，若情況嚴重或持續一段時間，請告知醫師，讓醫師為您調整藥量或使用其他類型的戒菸輔助劑。使用尼古清戒菸貼片期間，請勿同時使用其他含尼古丁之產品，以免造成尼古丁過量。使用尼古清戒菸貼片時，請避免貼在皮膚破損處，且每片貼片僅能使用一次，不可重複使用。使用尼古清戒菸貼片時，請依照醫師指示及說明書使用，一般建議每天貼一片，於睡前貼上，並於早上起床後移除。</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>不可以。若您已連續三天未解便，則須停用本藥，並洽詢醫師。</t>
+          <t>若您曾對尼古丁過敏或是懷孕、正在哺乳，請告知您的醫師您正服用任何其它藥物，包括非處方藥及天然療法產品，也務必讓您的醫師知道依照醫師指示正確使用藥品，未經醫師評估，請勿自行更改劑量或停藥。</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Diclofenac:這個藥是治什麼症狀的？</t>
+          <t>Nicotine: 我爸有心臟疾病用這個會有影響嗎?</t>
         </is>
       </c>
       <c r="C46" t="n">
         <v>2</v>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>非類固醇抗發炎藥(NSAID)，適用於類風濕性關節炎、骨關節炎、及僵直性脊椎炎之症狀治療。</t>
+          <t>尼古丁對心血管系統有刺激作用，可能加重心臟病患之病情，因此心臟病患使用時須小心。</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>這個藥是消炎止痛劑，用於緩解關節炎、扭傷、拉傷等引起的疼痛與發炎。</t>
+          <t>尼古丁對心血管系統有刺激作用，可能加重心臟疾病患者的症狀，如心絞痛、心律不整等。因此，心臟疾病患者使用尼古丁替代療法時應謹慎，最好在醫師監督下使用。</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>適用於緩解成人及小孩(6歲以上)因急性的局部關節/肌肉損傷所引起之疼痛。適用於緩解成人及青少年(16歲以上)因關節炎而產生的疼痛。適用於治療成人及小孩(6歲以上)的日光性角化症。</t>
+          <t>若您父親曾因心臟方面的原因而接受治療，建議您告知醫師，由醫師評估是否適合使用此產品。若有任何疑問或出現可能與心臟有關的症狀(如胸悶、胸痛等)，請儘速就診。</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Tolnaftate:當使用這個藥品，我該注意什麼?</t>
+          <t>Simethicone: 我小孩吃了好幾天了，作用不大，有更有效的藥嗎?</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
         <v>1</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>1.此藥僅供外用，且不可用於眼睛或黏膜。2.對此藥過敏者禁止使用。3.懷孕及授乳婦女不建議使用。4.使用後若出現皮膚刺激或過敏反應時，應停止使用。</t>
+          <t>本藥僅適用於消化不良及胃部不適感、脹氣、脹滿、打嗝、腹痛等症狀之對症治療，若您的小孩服藥後效果不佳，建議您帶他回診讓醫師評估是否適合改用其他藥物。</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>使用 Tolnaftate 時，請遵照醫師指示進行，並注意個人衛生習慣。</t>
+          <t>如果您的小孩已經持續使用Simethicone數天，但沒有明顯改善，建議您帶孩子就醫，由醫師評估是否需要調整藥物或進行其他治療。</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>若您屬於以下情況，請告知您的醫師：懷孕、計畫懷孕、正在母乳餵養嬰幼兒、計劃給孩子喂食此藥、已知對此藥過敏、有心律不整的情形等。您可能會感到頭暈或昏厥，所以如果您需要駕車或者操作機械設備，一定要小心。服藥期間需定期監測血液中的膽固醇含量。若您有任何疑問，請詢問醫生或藥師。</t>
+          <t>如果您的寶寶已經持續服用了數日但效果不佳，這可能是因為症狀變化較小或是其他因素影響治療結果。對於腹瀉、嘔吐等消化道問題，除了Simethicone外還有一些其他的療法治療效果可能會更好。具體來說，針對不同病因引起的相關症狀，如感染性腹瀉需抗感染治療、功能性腹痛則以調節腸蠕動及改善消化不良為主。此外，若是由食物過敏引起之症状，應避免食用致病的食物。若您對現有的治療方式感到疑問或者希望尋求更多幫助，建議您向醫生諮詢，以便獲得適合您孩子的個別化診斷與處方。</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Nicotine: 我爸有心臟疾病用這個會有影響嗎?</t>
+          <t>Amorolfine（Loceryl Nail Lacquer）:灰指甲擦了兩個月都沒好，是不是沒效？還要擦多久？</t>
         </is>
       </c>
       <c r="C48" t="n">
         <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>尼古丁對心血管系統有刺激作用，可能加重心臟病患之病情，因此心臟病患使用時須小心。</t>
+          <t>治療灰指甲通常需要較長時間，一般建議治療至少6個月以上。因此，您目前使用兩個月並未見療效，這可能是正常情況。請繼續按照醫師指示進行治療，不要自行停藥或更改劑量。</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>若您有心臟方面疾病，建議您在使用本藥前先告知醫師，由醫師評估是否適合使用。</t>
+          <t>治療灰指甲通常需要較長時間，一般建議至少使用6-12個月。因此，僅兩個月的治療可能尚未達到療效。建議持續按照醫師指示進行治療，並定期回診評估治療效果。</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>若您父親曾發生過心室性心搏过速或其他心室性異常心跳的情形,則應小心使用莫西沙星。</t>
+          <t>根據您所提供的信息，如果已經用了兩個月還沒有改善的話，建議您回診告知醫師，讓醫師幫忙評估是否適合繼續當前的治療方式或是需更換其他的治疗方法。</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Amorolfine:我該如何儲存這個藥品?</t>
+          <t>Chlorhexidine:我該如何儲存這個藥品?</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2091,17 +2089,17 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>室溫控制下保存。</t>
+          <t>室溫下存放。請放在小孩拿不到的地方，以免誤食造成危險。</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Hydrotalcite: 小孩吃了症狀沒變好，藥送醫嗎還是換個藥?</t>
+          <t>Fluticasone: 肝功能有異常的兒童劑量藥多少?</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -2115,337 +2113,339 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>請儘快帶小孩就醫，由醫師評估是否需調整藥量或改用其他藥物。</t>
+          <t>1.5 mg/天</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>請盡快就醫，由醫師評估是否需調整藥量或改用其他藥物。</t>
+          <t>對於肝功能有異常的兒童患者，使用Fluticasone的劑量應遵照醫師指示進行調整。一般來說，對於肝功能不全的成人患者，其劑量通常會減少；然而，對於兒童患者，其影響較少被研究，因此，對於兒童患者的用法和用量，請遵照醫師的指示。</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>如果孩子服用了足夠的劑量後，症狀仍然沒有改善，建議您帶孩子去看醫生，由醫師評估是否需要調整藥量或者改用其他藥物。</t>
+          <t>對於肝功能不全的小孩，沒有特定的建議劑量。但一般來說，如果孩子只有輕度到中等程度的肝臟問題，可能不需要改變劑量。然而，如果有任何疑問或者孩子的病情有所變化，應該立即聯絡醫生尋求幫助。</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cough Mixture 2:咳嗽糖漿喝了很想睡，白天還能繼續喝嗎？</t>
+          <t>Amorolfine:我該如何使用這個藥?</t>
         </is>
       </c>
       <c r="C51" t="n">
         <v>2</v>
       </c>
       <c r="D51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E51" t="n">
         <v>1</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>可以，但請注意白天服用此藥後若感到嗜睡，請勿從事容易引起傷害的危險活動，如開車、操作機械等。</t>
+          <t>遵照醫師指示使用。</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>可以，但請注意白天服用後的嗜睡情況，如有需要可調整服藥時間。</t>
+          <t>遵照醫師指示使用。通常建議每週使用一次，塗抹於患部，並持續塗抹直到藥膏乾燥。</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>可以，但若您服用後感到非常困倦，建議您於睡前服用此藥，以避免影響您的日常生活。</t>
+          <t>每日一次以手指尖輕柔地點滴於受感染部位(通常為指(趾)甲)，每週至少使用兩次，連續治療六個月以上。</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Duratears:我肝腎功能不好，可以使用嗎？</t>
+          <t>Minoxidil: 多久能開始有成效?</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D52" t="n">
         <v>2</v>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>若您有肝腎功能不全的情形，請告知您的醫師，由醫師評估是否適合使用。</t>
+          <t>一般在治療2-3週後可開始看到效果，6-8週後可看到明顯改善。</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>若您有肝腎功能障礙，請告知您的醫師，我們會依照您的情況調整劑量。</t>
+          <t>通常在使用後約4週可以看到初步效果，但完整的治療效果可能需要持續使用6個月以上。</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>若您有嚴重的肝臟疾病或腎臟疾病，請告知您的醫師，由醫師評估是否適合使用此藥。</t>
+          <t>通常在連續治療約4個月後可以看到頭髮生長的效果。</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Duratears: 皮膚好像熱熱的，正常嗎?</t>
+          <t>Fluticasone（Flixonase）:鼻噴劑症狀改善後，還需要每天噴嗎？會不會有依賴性？</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>2</v>
       </c>
       <c r="D53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>使用後可能會有眼睛灼熱感或刺痛感，此症狀通常在15分鐘內消失。</t>
+          <t>即使症狀改善，仍需每天使用，以維持預防作用。並無成癮性。</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>使用Metrogel凝膠後，可能會有局部熱感、灼熱感或刺痛感，這都是常見的副作用。但如果您的皮膚出現嚴重的紅腫、水泡或脫皮等現象，請立即停藥並就醫。</t>
+          <t>即使症狀改善，仍應持續按照醫師指示使用，以維持治療效果。通常建議每日一次，持續使用。使用後可能會有暫時性的鼻腔刺激感，但不影響使用。長期使用可能會有局部副作用，如鼻腔感染、鼻出血等，但一般停藥後即可恢復。並無明確證據顯示此藥會產生依賴性。</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>是的，您可能會感到局部暖暖的或有輕微的燒灼感，這都是正常的現象。但若您出現嚴重的過敏反應如呼吸困難、喉嚨緊繃等症狀時，請立即停藥就醫。</t>
+          <t>即使您的哮喘症狀得到緩解，您仍然應該按照醫生指示繼續使用Flixonase。突然停藥可能會導致嚴重的呼吸問題再次發生。這不是對身體產生依賴性的結果，而是因為持續治療的必要性。</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Nicotine（Nicorette／Smokfree）:我抽菸的同時使用戒菸口香糖，這樣會不會有問題？</t>
+          <t>Nicotine: 我照顧的老人正在用這個藥有甚麼我要注意的嗎?</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D54" t="n">
         <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>不建議在抽菸時使用戒菸口香糖，因為這兩種產品都是為了緩解戒斷症狀而設計的，如果同時使用可能會造成過度刺激。</t>
+          <t>1. 請勿讓其他人使用您的藥品。2. 若您對尼古丁過敏或懷孕，請告知醫師。3. 若您正在服用下列藥品，請告知醫師：抗潰瘍劑、抗凝血劑、降血糖藥、制酸劑、避孕藥、抗癲癇藥、抗憂鬱劑、抗心律不整劑、β-阻斷劑、甲狀腺素、利尿劑、止痛劑、止咳劑、緩瀉劑、鈣離子阻斷劑。4. 若您有肝臟疾病、糖尿病、高血壓、心臟病、胃潰瘍、胃食道逆流、腎臟疾病、甲狀腺機能亢進、癲癇、青光眼、氣喘、肺氣腫、心律不整、中風、心肌梗塞、胸痛、心悸、頭痛</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>尼古丁口香糖與本藥物併用可能會降低本藥物的療效。</t>
+          <t>尼古丁貼片可能會引起皮膚過敏反應，如紅腫、發癢等症狀，若發生此情況請告知醫師。尼古丁貼片可能會影響其他藥品的效果，因此請告知醫師您正在服用的藥品。尼古丁貼片可能會引起心跳加速、頭痛、噁心等症狀，若發生此情況請告知醫師。尼古丁貼片可能會對未出生的胎兒造成傷害，因此懷孕婦女不建議使用。</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>可以一起服用，但建議不要咀嚼太快，以免影響尼古丁之吸收。</t>
+          <t>如果您是幫助您的家人服藥，建議您留意以下事項:
+1. 若您的家人生氣、焦慮、頭暈、嘔吐等症狀時，可能是戒斷症狀或是副作用產生，請提醒他依照醫師指示服用此藥。
+2. 避免讓您的家人同時服用其他可能增加低血壓之藥物(如抗凝血劑)，以免造成出血的情形。</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Crotamiton: 推薦我用這個藥的原因是甚麼?</t>
+          <t>Urea:為什麼我要使用這個藥?</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E55" t="n">
         <v>1</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>治療疥瘡、陰蝨感染。</t>
+          <t>此藥用於治療高血漿尿素氮症，通常發生於腎臟病患者。</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>此藥用於治療濕疹、牛皮癬、蕁麻疹、皮膚炎、燒傷、蟲咬、疥瘡、汗斑等皮膚疾病。</t>
+          <t>尿素軟膏用於治療皮膚角化症，如魚鳞狀皮膚症、掌蹠性角化症、乾癬等。</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>治療濕疹性皮膚炎、蕁麻疹及尋常型痤瘡。</t>
+          <t>此藥通常被用作外用軟膏、乳液或其他形式的局部治療。它具有去角質作用，可以幫助去除表層皮膚細胞，對於某些類型的濕疹、牛皮癬等皮膚疾病有療效。此外，還可以用於處理嚴重燒傷後留下的疤痕。</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Crotamiton: 藥效可以持續多久?</t>
+          <t>Betamethasone: 如果一直沒使用完，可以放多久還能用?</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>本藥通常建議每日使用一次即可達到療效，但若為了增加藥效，可於睡前再塗抹一次。</t>
+          <t>未開封前可存放於室溫下(30℃以下)，避免陽光直射。一旦打開包裝或放入冰箱，需在6週內使用完。</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Naproxen屬於非類固醇抗發炎藥(NSAID)，具有抗發炎、止痛、解熱的作用。Naproxen的半衰期約4至6小時，因此每6至8小時需服用一次。</t>
+          <t>未開封的外用劑可於室溫下存放三個月。超過三個月未使用完，請丟棄。</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>通常一天一次即可。但若有特殊情況需要更頻繁使用的，建議詢問醫師指示。</t>
+          <t>室溫下保存不超過一個月。</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cough Mixture:為什麼我要使用這個藥?</t>
+          <t>Hydrotalcite（NACID）:胃不舒服想吃 NACID，但我還在吃其他慢性病藥，可以一起服用嗎？</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>本藥品是化痰劑，可以幫助排痰。</t>
+          <t>不可以，請先告知醫師您正在服用的藥物，由醫師評估是否適合併服。</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>這個藥品主要是用來治療類風濕性關節炎、骨關節炎。</t>
+          <t>請先告知您的醫師，由醫師評估是否適合同時服用。</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Flixonase可以緩解過敏性鼻炎引起的相關症狀。</t>
+          <t>若您同時有其他的慢性病正在服藥，請告知您的醫師，由醫師評估是否適合併服此藥。若需併服其他藥品，則至少間隔兩小時以上再服用此藥，以避免影響藥效。</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Povidone Iodine:這個藥有用吃的嗎?效果會不會比較好?</t>
+          <t>Crotamiton: 藥效可以持續多久?</t>
         </is>
       </c>
       <c r="C58" t="n">
         <v>2</v>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E58" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Povidone Iodine並無口服劑型，僅有外用劑型。</t>
+          <t>本藥通常建議每日使用一次即可達到療效，但若為了增加藥效，可於睡前再塗抹一次。</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Povidone Iodine 是外用消毒劑，通常用於手部消毒或外科手術前的皮膚消毒。它不是口服藥物，所以不能吃下肚來治療感染。</t>
+          <t>Crotamiton 通常建議每 8 小時使用一次，連續使用 7 天。因此，其藥效可以持續約 8 小時左右。</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>不可以用吃的方式服用，只能外用。</t>
+          <t>治療期間每日塗抹，停藥後可維持效果約一天。</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Minoxidil: 多久能開始有成效?</t>
+          <t>Diclofenac:我該如何使用這個藥?</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D59" t="n">
         <v>3</v>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>一般在治療2-3週後可開始看到效果，6-8週後可看到明顯改善。</t>
+          <t>請遵照醫師指示及藥袋上之說明服用此藥藥期間請保留藥袋，以便即時獲取藥品資訊便症狀改善/病情穩定，仍應持續按照醫師指示服藥非醫師特別指示，此藥飯前或飯後服用皆可。</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>通常在治療初期，可能會出現頭髮脫落現象，但隨著治療持續，頭髮會逐漸再生長。一般來說，治療約2至3個月後，可以開始看到頭髮再生長的效果。</t>
+          <t>請遵照醫師指示及藥袋上之說明服用此藥。一般建議劑量為每次50~100mg，每日2~3次。</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>通常需要持續使用數周至數月才能看到明顯的效果。</t>
+          <t>請依照醫師指示及個人需要調整用量，但每次使用的最小間隔至少需超過四小時以上。您可自行決定是否以冷敷方式降低局部之不適感。</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Miconazole: 糖尿病患者有甚麼要注意的嗎?</t>
+          <t>Acetaminophen（Anti-phen）:我吃了 Anti-phen 退燒，但效果不好，可以自己增加劑量嗎？</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D60" t="n">
         <v>2</v>
@@ -2455,31 +2455,31 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>使用本劑可能會引起低血糖，若同時服用降血糖藥物者，請告知醫師，以利評估您的治療方案。</t>
+          <t>不可以，請回診讓醫師評估。</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>使用米康唑治療期間，糖尿病患者的血糖控制可能會受到影響。因此，建議糖尿病患者在使用米康唑期間，定期監測血糖值，並與醫師討論 Adjustment of antidiabetic therapy may be necessary during treatment with micafungin. Regular monitoring of blood glucose is recommended.</t>
+          <t>不可以自行增加劑量，請回診與醫師討論。</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>糖尿病患服用此藥可能會造成血糖控制困難，因此須密切追蹤其血糖值。</t>
+          <t>不可以自行增額外需要服藥的情況下，請回診讓醫師評估是否可調高劑量，切勿擅自增加劑量。</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>66</v>
+        <v>23</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ibuprofen:這藥是怎麼運作的</t>
+          <t>Betamethasone:我該如何儲存這個藥品?</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D61" t="n">
         <v>1</v>
@@ -2489,200 +2489,197 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>布洛芬是一種非類固醇抗發炎藥(NSAID)，具有解熱、止痛、抗發炎作用。</t>
+          <t>室溫下緊密容器儲存。避免直接日照、熱、和溼氣。</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Ibuprofen屬於非類固醇抗發炎藥(NSAID)，它通過抑制體內前列腺素的合成，而達到抗發炎、止痛、退燒的效果。</t>
+          <t>室溫下儲存。避免直接暴露於日照、熱、和溼氣之下。請放在小孩拿不到處，以免誤食造成危險。</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>非甾體抗發炎藥(NSAID)，具有解熱、止痛、抗發炎作用。</t>
+          <t>請存放於25°C(77°F)以下。遠離火源、明火或高溫。請勿置於陽光直射處。</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Diclofenac:小朋友或老人家使用時需要特別注意什麼？</t>
+          <t>Amorolfine:我該如何儲存這個藥品?</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D62" t="n">
         <v>1</v>
       </c>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>1. 有肝臟或腎臟疾病的小朋友，不建議使用。2. 有胃潰瘍或腸胃道出血問題的小朋友，不建議使用。3. 有嚴重氣喘、高血壓、心臟病、糖尿病、肝臟或腎臟疾病的老年患者，請先告訴醫師。</t>
+          <t>室溫下緊密容器儲存。避免直接日照、熱、和溼氣。</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>對於小朋友或老人家，使用Diclofenac時需要特別注意以下幾點：
-1. 對於小童，尤其是嬰兒，長期使用Diclofenac可能會影響骨骼生長，因此僅在必要時才可使用，且應遵照醫師指示。
-2. 老人因肝腎功能可能較差，使用Diclofenac時可能會增加不良反應的風險，因此也應遵照醫師指示，必要時調整劑量。
-3. 所有年齡層的患者，在使用Diclofenac期間，都應定期監測肝腎功能，以確保安全。</t>
+          <t>室溫下儲存。避免直接暴露於日照、熱、和溼氣之下。</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>為了避免副作用發生，尤其是肝腎功能方面，因此小童及老人須小心使用。</t>
+          <t>室溫下避光保存。</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>我口腔潰瘍發炎可以用什麼藥?</t>
+          <t>Tolnaftate:當使用這個藥品，我該注意什麼?</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>可以使用含有類固醇的漱口水或口腔凝膠，如：Orabas 1000、Orabas 250、Orabas 500、Orabas 1000 forte、Orabas 1000 gel、Orabas 250 gel、Orabas 500 gel、Orabas 1000 forte gel。</t>
+          <t>1.此藥僅供外用，且不可用於眼睛或黏膜。2.對此藥過敏者禁止使用。3.懷孕及授乳婦女不建議使用。4.使用後若出現皮膚刺激或過敏反應時，應停止使用。</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>口腔潰瘍發炎通常建議使用局部消炎止痛藥，例如口腔溃疡專用凝膠，或者含漱液如氯己定含漱液等。但您如果是因低血壓引起症狀，則需遵照醫師指示服用相關藥品，不建議自行更改藥品或治療方式。</t>
+          <t>對此成份過敏者禁止使用；請勿長期連續使用果有懷孕、哺乳、肝腎疾病或有服用其他藥物應告知醫師用此藥後若出現過敏反應如皮膚紅腫、發癢、呼吸困難、喉嚨緊縮等症狀時，須立即停藥並就醫用此藥後若出現頭暈、昏眩、視力模糊等症狀時，須避免從事危險性工作如開車、操作機械等。</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>可以使用含有類固醇成分之漱口水，如：Betadine Anti-Inflamatory Oral Rinse(百多邦消腫漱口水)，以減輕癢感及紅腫現象；另外也可以局部涂抹類固醇軟膏，如：Diprosone Ointment(迪普松乳膏)於患部，但皆應遵照醫師指示使用。</t>
+          <t>若您有下列情況，請告知您的醫師：懷孕、計畫懷孕、哺乳、曾對此藥過敏、其他疾病(如心臟血管疾病、腎臟疾病等)您可能會感到刺痛感或是灼熱感，這都是正常現象，但如果您覺得不適感持續數小時以上，則需立即停藥並回診就醫。</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Ibuprofen: 可以和Diclofenac同時使用嗎?</t>
+          <t>Diclofenac:這個藥是治什麼症狀的？</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>不可以，兩種藥物都屬於非類固醇抗發炎藥(NSAID)，不建議同時服用。</t>
+          <t>非類固醇抗發炎藥(NSAID)，適用於類風濕性關節炎、骨關節炎、及僵直性脊椎炎之症狀治療。</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>不可以同時使用，因為可能會增加出血的危險性。</t>
+          <t>非類固醇抗發炎藥(NSAID)，具有解熱、止痛、抗發炎作用。可治療關節炎、風濕性關節炎、骨關節炎、急性痛風性關節炎、肌肉痙攣、經期疼痛。</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>不可以同時使用，因為可能增加出血風險。</t>
+          <t>適用於緩解下列情況之疼痛及發炎現象。1. 閂可舒軟膏：適用於緩解成人及兩歲以上孩童因急性和慢性關節、肌肉損傷所引起之疼痛及發炎現象。2. 閘康錠：適用於緩解成人及兩歲以上孩童因急性和慢性關節、肌肉損傷所引起之疼痛及發炎現象。3. 閡安膜衣錠：適用於緩解成人及兩歲以上孩童因急性和慢性關節、肌肉損傷所引起之疼痛及發炎現象。4. 閣能散懸液：適用於緩解成人及兩歲以上孩童因急性和慢性關節、肌肉損傷所引起之疼痛及發炎現象。</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Hydrocortisone:我該如何使用這個藥?</t>
+          <t>Diclofenac:小朋友或老人家使用時需要特別注意什麼？</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>遵照醫師指示使用。</t>
+          <t>1. 有肝臟或腎臟疾病的小朋友，不建議使用。2. 有胃潰瘍或腸胃道出血問題的小朋友，不建議使用。3. 有嚴重氣喘、高血壓、心臟病、糖尿病、肝臟或腎臟疾病的老年患者，請先告訴醫師。</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>請依照醫師指示使用，通常一天使用兩次，每次使用一滴。</t>
+          <t>對小孩及老人而言，使用非固醇類抗發炎藥可能較容易出現副作用，因此請依照醫師指示用藥，並密切觀察反應。</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>請依照醫師指示使用，通常每日一次，每次一粒(約1克)，可溶於水後經由口腔黏膜投予。</t>
+          <t>對於小童及老人，因可能會影響其肝功能或腎功能，故應小心監測其副作用。</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Duratears:這藥可以幹嗎?</t>
+          <t>Minoxidil:我該如何儲存這個藥品?</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Duratears用於治療乾眼症。</t>
+          <t>室溫下儲存。</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Duratears用於治療細菌所引起的感染。</t>
+          <t>室溫下儲存。</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Duratears是一種治療乾眼症的滴眼液，它含有兩種成分：人工淚水和抗潰瘍病毒藥物。人工淚水部分可緩解眼睛乾澀不適感；而抗潰瘍病毒藥物則具有殺菌作用，能減少眼部細菌感染。因此，Duratears對於因乾燥引起的眼部刺激及炎症具有良好的療效。</t>
+          <t>請儲存在室溫下，避免高溫及曝曬陽光。請存放於兒童拿不到的地方，以免誤食造成危險。</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Povidone Iodine:這個藥要怎麼使用效果最好？一天要用幾次、用多久？</t>
+          <t>Povidone Iodine: 孩子誤食了，會需要做什麼嗎?</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -2696,153 +2693,153 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>本藥品為外用消毒劑，通常建議每日使用2-3次，直到感染症狀消失。</t>
+          <t>若孩子誤食了，請立即就醫。</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Povidone Iodine並非本品的使用方法，可能是您想問的是本品的使用方法。本品需由醫師處方使用，通常在口腔黏膜下注射，每天一次，連續使用7天。</t>
+          <t>如果孩子誤食了碘酒，通常情況下不需要特別治療，因為口服少量碘酒對身體影響不大。但是，如果孩子出現任何異常反應，如呼吸困難、喉嚨腫脹、皮膚紅腫、噁心、嘔吐、腹瀉、頭痛、眩暈、心悸等，請立即就醫。</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>根據 Lexidrug 提供的信息，此藥通常用作外用消毒劑，如口腔漱口水或局部涂抹。一般來說，成人每日可使用數次，但總量應控制在每日少於 4 次，每次 10毫升。对于其他用途，请遵循醫生指示。</t>
+          <t>如果孩子誤服了povidone碘，應立即就診。一般來說，小劑量可能不會引起嚴重問題，但為了安全起見，仍需由醫師評估。若大量服用，可能會出現胃腸道刺激症狀如嘔吐、腹瀉等，必要時須進行洗胃或其他對癢處理措施。</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Sodium phosphate:使用這個藥品有可能會出現那些副作用?</t>
+          <t>Hydrotalcite: 小孩吃了症狀沒變好，藥送醫嗎還是換個藥?</t>
         </is>
       </c>
       <c r="C68" t="n">
         <v>1</v>
       </c>
       <c r="D68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>腹痛、腹脹、噁心、嘔吐、頭痛、暈眩、皮膚過敏。</t>
+          <t>請儘快帶小孩就醫，由醫師評估是否需調整藥量或改用其他藥物。</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>使用這個藥品可能會出現噁心、嘔吐、瀉肚及過敏反應等副作用。</t>
+          <t>如果孩子服用Hydrotalcite後，症狀沒有改善，建議您帶孩子去看醫生，由醫師評估是否需要調整藥量或換藥。</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>服用此藥可能會造成消化不良、食慾不振、脹氣、腹痛、便祕、腹部痙攣等現象。若您有任何疑問或者情況持續惡化的時候，請立即告知您的醫師。</t>
+          <t>如果孩子服用了建議的劑量後，症狀仍然沒有改善或者病情惡化，應儘快就診。可能需要評估是否適合繼續當前療程或是改用其他藥物。</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Dextromethorphan:我正在吃其他藥或保健食品，可以一起使用嗎？</t>
+          <t>Nicotine:為什麼我要使用這個藥?</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E69" t="n">
         <v>1</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>若您正在服用其他藥品，請先告知醫師或藥師，以確保安全。</t>
+          <t>尼古丁口錐可幫助戒除尼古丁成癮，減少抽菸次數或戒除抽菸。</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>若您正在服用其他藥品或保健食品，請務必告知您的醫師，以確保安全使用。</t>
+          <t>尼古丁貼片用於戒菸。尼古丁咀嚼錠用於治療注意力缺損過動症(ADHD)。尼古丁鼻噴霧劑用於治療注意力缺損過動症(ADHD)。尼古丁吸入器用於治療注意力缺損過動症(ADHD)。尼古丁溶液用於治療注意力缺損過動症(ADHD)。</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>若您同時服用了dextromethorphan，可能會增加副作用的產生，建議避免同時服用。</t>
+          <t>SmokFree Nicotine Patch 是一種尼古丁替代療法(NRT)，適用於輔助戒煙。它通過釋放小量的尼古丁到體內，以減輕戒煙帶來的不適感及渴求感。</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Simethicone: 我小孩吃了好幾天了，作用不大，有更有效的藥嗎?</t>
+          <t>Duratears: 皮膚好像熱熱的，正常嗎?</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E70" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>本藥僅適用於消化不良及胃部不適感、脹氣、脹滿、打嗝、腹痛等症狀之對症治療，若您的小孩服藥後效果不佳，建議您帶他回診讓醫師評估是否適合改用其他藥物。</t>
+          <t>使用後可能會有眼睛灼熱感或刺痛感，此症狀通常在15分鐘內消失。</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>對于胃脹氣，除了使用Simethicone外，還可以考慮使用其他消化酶製劑，如胰酶、膽汁酸等。此外，調整飲食習慣，避免食用容易产气的食物，如豆類、牛奶等，也有助於改善胃脹氣的問題。</t>
+          <t>使用Duratears眼藥水後可能會出現暫時性的眼部灼熱感、刺痛感、搔癢感等不適感，這些症狀通常在數分鐘內消失。若症狀持續數天或加劇，請立即停藥並就醫。</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>可以考慮其他消化酵素產品，如Pancreatin等；若屬於胃腸蠕動不順問題，可考慮使用甲氧氯普胺錠。</t>
+          <t>是正常的。您若對此有疑問，建議詢問您的醫師。</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Hydrotalcite（NACID）:胃不舒服想吃 NACID，但我還在吃其他慢性病藥，可以一起服用嗎？</t>
+          <t>Povidone Iodine:優碘是不是擦越多越好？傷口每天都要消毒嗎？</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D71" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>不可以，請先告知醫師您正在服用的藥物，由醫師評估是否適合併服。</t>
+          <t>擦太多會使皮膚過於乾燥，且對皮膚有刺激性。傷口每天不需要消毒，但若有分泌物或感染時則需適當清潔。</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>不可以，請先告知您的醫師，由醫師評估是否可同時服用。</t>
+          <t>使用優碘時，建議僅塗抹薄薄一層即可，過量使用可能會造成皮膚刺激。傷口是否需要每天消毒，應遵照醫師指示。一般而言，清潔傷口後，可依需要進行必要的消毒；若傷口已經癒合，則不需再行消毒。</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>不可以直接吞服此顆粒劑，需以足量冷開水混合均勻後再口服。若您同時正在服用其他藥品，則兩種藥品須分別服用，間隔至少一小時以上。</t>
+          <t>不是的，擦拭次數及用量應依照醫師指示進行，通常建議一天四次即可。</t>
         </is>
       </c>
     </row>

</xml_diff>